<commit_message>
Rebrand: Marius FX -> MS Prime (logo, titles/meta/OG, JSON-LD org, manifest, icons, og-image, journal templates + exports, RO/EN/ES/PT). Person Marius, URLs, email, Telegram, storage keys unchanged. Revert: tag pre-msprime
</commit_message>
<xml_diff>
--- a/downloads/jurnal-tranzactionare-marius-fx.xlsx
+++ b/downloads/jurnal-tranzactionare-marius-fx.xlsx
@@ -784,7 +784,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Jurnal de tranzacționare — Marius FX</t>
+          <t>Jurnal de tranzacționare — MS Prime</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3872,7 +3872,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CMarius FX — Jurnal de tranzacționare · pagina &amp;P din &amp;N</oddFooter>
+    <oddFooter>&amp;CMS Prime — Jurnal de tranzacționare · pagina &amp;P din &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>